<commit_message>
Actualizado el generador de correos y WhatsApp en app.py con plantillas institucionales de Padrinos GGP
</commit_message>
<xml_diff>
--- a/data/Matriz_Seguimiento_Proyectos_Cesar.xlsx
+++ b/data/Matriz_Seguimiento_Proyectos_Cesar.xlsx
@@ -412,7 +412,7 @@
     <t>Ramón Alberto Rubio Durango</t>
   </si>
   <si>
-    <t>Milton Alexis Olaya Santamaria</t>
+    <t>Milton Olaya Santamaría</t>
   </si>
   <si>
     <t>Katherine Mora Rosado</t>
@@ -424,7 +424,7 @@
     <t>Felix Antonio Henao Casanova</t>
   </si>
   <si>
-    <t>Alexander Kowoll</t>
+    <t>Alexander Botello López</t>
   </si>
   <si>
     <t>José Reinel Contreras Yaruro</t>
@@ -433,7 +433,7 @@
     <t>Robeiro Muñoz Pérez</t>
   </si>
   <si>
-    <t>Yader José Claro Castro</t>
+    <t>Yoly Margarita Ruedas León</t>
   </si>
   <si>
     <t>Emiro Cañizares Plata</t>

</xml_diff>